<commit_message>
Merge regimes; README, WALKTHROUGH, RESULTS; untrack bulky labelled CSVs
</commit_message>
<xml_diff>
--- a/results/regimes/regimes.xlsx
+++ b/results/regimes/regimes.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="regime_summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="episode_coverage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="transition_hmm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="transition_threshold" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="spread_stats" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="rolling_corr_tail" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="corr_changes_r0" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="corr_changes_r1" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="corr_changes_r2" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="corr_levels_r0" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="corr_levels_r1" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="corr_levels_r2" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="provenance" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regime_summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="episode_coverage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="transition_hmm" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="transition_threshold" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="spread_stats" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rolling_corr_tail" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="corr_changes_r0" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="corr_changes_r1" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="corr_changes_r2" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="corr_levels_r0" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="corr_levels_r1" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="corr_levels_r2" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="provenance" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,13 +32,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,7 +52,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -57,13 +60,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -433,39 +447,39 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>regime</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>days</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>share_pct</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>first_date</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>last_date</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>mean_stress_score</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
@@ -492,7 +506,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="n">
@@ -519,7 +533,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="n">
@@ -560,49 +574,49 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>1y-3m</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>2y-1y</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>5y-2y</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>10y-5y</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>5y-1y</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>fly 2*1y-3m-2y</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>fly 2*2y-1y-5y</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>fly 2*5y-2y-10y</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>1y-3m</t>
         </is>
@@ -633,7 +647,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>2y-1y</t>
         </is>
@@ -664,7 +678,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>5y-2y</t>
         </is>
@@ -695,7 +709,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>10y-5y</t>
         </is>
@@ -726,7 +740,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>5y-1y</t>
         </is>
@@ -757,7 +771,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>fly 2*1y-3m-2y</t>
         </is>
@@ -788,7 +802,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>fly 2*2y-1y-5y</t>
         </is>
@@ -819,7 +833,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>fly 2*5y-2y-10y</t>
         </is>
@@ -864,49 +878,49 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>1y-3m</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>2y-1y</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>5y-2y</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>10y-5y</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>5y-1y</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>fly 2*1y-3m-2y</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>fly 2*2y-1y-5y</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>fly 2*5y-2y-10y</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>1y-3m</t>
         </is>
@@ -937,7 +951,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>2y-1y</t>
         </is>
@@ -968,7 +982,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>5y-2y</t>
         </is>
@@ -999,7 +1013,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>10y-5y</t>
         </is>
@@ -1030,7 +1044,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>5y-1y</t>
         </is>
@@ -1061,7 +1075,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>fly 2*1y-3m-2y</t>
         </is>
@@ -1092,7 +1106,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>fly 2*2y-1y-5y</t>
         </is>
@@ -1123,7 +1137,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>fly 2*5y-2y-10y</t>
         </is>
@@ -1168,49 +1182,49 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>1y-3m</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>2y-1y</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>5y-2y</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>10y-5y</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>5y-1y</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>fly 2*1y-3m-2y</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>fly 2*2y-1y-5y</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>fly 2*5y-2y-10y</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>1y-3m</t>
         </is>
@@ -1241,7 +1255,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>2y-1y</t>
         </is>
@@ -1272,7 +1286,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>5y-2y</t>
         </is>
@@ -1303,7 +1317,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>10y-5y</t>
         </is>
@@ -1334,7 +1348,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>5y-1y</t>
         </is>
@@ -1365,7 +1379,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>fly 2*1y-3m-2y</t>
         </is>
@@ -1396,7 +1410,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>fly 2*2y-1y-5y</t>
         </is>
@@ -1427,7 +1441,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>fly 2*5y-2y-10y</t>
         </is>
@@ -1472,12 +1486,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>key</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
@@ -1606,49 +1620,49 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>episode</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>start</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>end</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>days</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>elevated_share_pct</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>stressed_share_pct</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>detected</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>in_scope</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -1683,7 +1697,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -1718,7 +1732,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -1753,7 +1767,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -1802,18 +1816,18 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="n">
+      <c r="B1" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="C1" t="n">
+      <c r="C1" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D1" t="n">
+      <c r="D1" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
@@ -1827,7 +1841,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="n">
@@ -1841,7 +1855,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="n">
@@ -1869,24 +1883,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>to_0</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>to_1</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>to_2</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>from_0</t>
         </is>
@@ -1902,7 +1916,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>from_1</t>
         </is>
@@ -1918,7 +1932,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>from_2</t>
         </is>
@@ -1948,49 +1962,49 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>mean</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>std</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>min</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>75%</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>max</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>1y-3m</t>
         </is>
@@ -2021,7 +2035,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>2y-1y</t>
         </is>
@@ -2052,7 +2066,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>5y-2y</t>
         </is>
@@ -2083,7 +2097,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>10y-5y</t>
         </is>
@@ -2114,7 +2128,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>5y-1y</t>
         </is>
@@ -2145,7 +2159,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>fly 2*1y-3m-2y</t>
         </is>
@@ -2176,7 +2190,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>fly 2*2y-1y-5y</t>
         </is>
@@ -2207,7 +2221,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>fly 2*5y-2y-10y</t>
         </is>
@@ -2252,29 +2266,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>corr(2y-1y,5y-2y)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>corr(2y-1y,10y-5y)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>corr(2y-1y,fly 2*2y-1y-5y)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>45939</v>
       </c>
       <c r="B2" t="n">
@@ -2288,7 +2302,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>45940</v>
       </c>
       <c r="B3" t="n">
@@ -2302,7 +2316,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>45944</v>
       </c>
       <c r="B4" t="n">
@@ -2316,7 +2330,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>45945</v>
       </c>
       <c r="B5" t="n">
@@ -2330,7 +2344,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>45946</v>
       </c>
       <c r="B6" t="n">
@@ -2344,7 +2358,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>45947</v>
       </c>
       <c r="B7" t="n">
@@ -2358,7 +2372,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>45950</v>
       </c>
       <c r="B8" t="n">
@@ -2372,7 +2386,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>45951</v>
       </c>
       <c r="B9" t="n">
@@ -2386,7 +2400,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>45952</v>
       </c>
       <c r="B10" t="n">
@@ -2400,7 +2414,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>45953</v>
       </c>
       <c r="B11" t="n">
@@ -2414,7 +2428,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>45954</v>
       </c>
       <c r="B12" t="n">
@@ -2428,7 +2442,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>45957</v>
       </c>
       <c r="B13" t="n">
@@ -2442,7 +2456,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>45958</v>
       </c>
       <c r="B14" t="n">
@@ -2456,7 +2470,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>45959</v>
       </c>
       <c r="B15" t="n">
@@ -2470,7 +2484,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>45960</v>
       </c>
       <c r="B16" t="n">
@@ -2484,7 +2498,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>45961</v>
       </c>
       <c r="B17" t="n">
@@ -2498,7 +2512,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>45964</v>
       </c>
       <c r="B18" t="n">
@@ -2512,7 +2526,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>45965</v>
       </c>
       <c r="B19" t="n">
@@ -2526,7 +2540,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>45966</v>
       </c>
       <c r="B20" t="n">
@@ -2540,7 +2554,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>45967</v>
       </c>
       <c r="B21" t="n">
@@ -2554,7 +2568,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>45968</v>
       </c>
       <c r="B22" t="n">
@@ -2568,7 +2582,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>45971</v>
       </c>
       <c r="B23" t="n">
@@ -2582,7 +2596,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>45973</v>
       </c>
       <c r="B24" t="n">
@@ -2596,7 +2610,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>45974</v>
       </c>
       <c r="B25" t="n">
@@ -2610,7 +2624,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" s="2" t="n">
         <v>45975</v>
       </c>
       <c r="B26" t="n">
@@ -2624,7 +2638,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" s="2" t="n">
         <v>45978</v>
       </c>
       <c r="B27" t="n">
@@ -2638,7 +2652,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="B28" t="n">
@@ -2652,7 +2666,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" s="2" t="n">
         <v>45980</v>
       </c>
       <c r="B29" t="n">
@@ -2666,7 +2680,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" s="2" t="n">
         <v>45981</v>
       </c>
       <c r="B30" t="n">
@@ -2680,7 +2694,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" s="2" t="n">
         <v>45982</v>
       </c>
       <c r="B31" t="n">
@@ -2694,7 +2708,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" s="2" t="n">
         <v>45985</v>
       </c>
       <c r="B32" t="n">
@@ -2708,7 +2722,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="B33" t="n">
@@ -2722,7 +2736,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="2" t="n">
         <v>45987</v>
       </c>
       <c r="B34" t="n">
@@ -2736,7 +2750,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>45989</v>
       </c>
       <c r="B35" t="n">
@@ -2750,7 +2764,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" s="2" t="n">
         <v>45992</v>
       </c>
       <c r="B36" t="n">
@@ -2764,7 +2778,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" s="2" t="n">
         <v>45993</v>
       </c>
       <c r="B37" t="n">
@@ -2778,7 +2792,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="B38" t="n">
@@ -2792,7 +2806,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" s="2" t="n">
         <v>45995</v>
       </c>
       <c r="B39" t="n">
@@ -2806,7 +2820,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="2" t="n">
         <v>45996</v>
       </c>
       <c r="B40" t="n">
@@ -2820,7 +2834,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" s="2" t="n">
         <v>45999</v>
       </c>
       <c r="B41" t="n">
@@ -2834,7 +2848,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" s="2" t="n">
         <v>46000</v>
       </c>
       <c r="B42" t="n">
@@ -2848,7 +2862,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" s="2" t="n">
         <v>46001</v>
       </c>
       <c r="B43" t="n">
@@ -2862,7 +2876,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" s="2" t="n">
         <v>46002</v>
       </c>
       <c r="B44" t="n">
@@ -2876,7 +2890,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" s="2" t="n">
         <v>46003</v>
       </c>
       <c r="B45" t="n">
@@ -2890,7 +2904,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="B46" t="n">
@@ -2904,7 +2918,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" s="2" t="n">
         <v>46007</v>
       </c>
       <c r="B47" t="n">
@@ -2918,7 +2932,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" s="2" t="n">
         <v>46008</v>
       </c>
       <c r="B48" t="n">
@@ -2932,7 +2946,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" s="2" t="n">
         <v>46009</v>
       </c>
       <c r="B49" t="n">
@@ -2946,7 +2960,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" s="2" t="n">
         <v>46010</v>
       </c>
       <c r="B50" t="n">
@@ -2960,7 +2974,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="2" t="n">
         <v>46013</v>
       </c>
       <c r="B51" t="n">
@@ -2974,7 +2988,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="B52" t="n">
@@ -2988,7 +3002,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="2" t="n">
         <v>46015</v>
       </c>
       <c r="B53" t="n">
@@ -3002,7 +3016,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="2" t="n">
         <v>46017</v>
       </c>
       <c r="B54" t="n">
@@ -3016,7 +3030,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="2" t="n">
         <v>46020</v>
       </c>
       <c r="B55" t="n">
@@ -3030,7 +3044,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" s="2" t="n">
         <v>46021</v>
       </c>
       <c r="B56" t="n">
@@ -3044,7 +3058,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" s="2" t="n">
         <v>46022</v>
       </c>
       <c r="B57" t="n">
@@ -3058,7 +3072,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" s="2" t="n">
         <v>46024</v>
       </c>
       <c r="B58" t="n">
@@ -3072,7 +3086,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" s="2" t="n">
         <v>46027</v>
       </c>
       <c r="B59" t="n">
@@ -3086,7 +3100,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="B60" t="n">
@@ -3100,7 +3114,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" s="2" t="n">
         <v>46029</v>
       </c>
       <c r="B61" t="n">
@@ -3114,7 +3128,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" s="2" t="n">
         <v>46030</v>
       </c>
       <c r="B62" t="n">
@@ -3128,7 +3142,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" s="2" t="n">
         <v>46031</v>
       </c>
       <c r="B63" t="n">
@@ -3142,7 +3156,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" s="2" t="n">
         <v>46034</v>
       </c>
       <c r="B64" t="n">
@@ -3156,7 +3170,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" s="2" t="n">
         <v>46035</v>
       </c>
       <c r="B65" t="n">
@@ -3170,7 +3184,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" s="2" t="n">
         <v>46036</v>
       </c>
       <c r="B66" t="n">
@@ -3184,7 +3198,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" s="2" t="n">
         <v>46037</v>
       </c>
       <c r="B67" t="n">
@@ -3198,7 +3212,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" s="2" t="n">
         <v>46038</v>
       </c>
       <c r="B68" t="n">
@@ -3212,7 +3226,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" s="2" t="n">
         <v>46042</v>
       </c>
       <c r="B69" t="n">
@@ -3226,7 +3240,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" s="2" t="n">
         <v>46043</v>
       </c>
       <c r="B70" t="n">
@@ -3240,7 +3254,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" s="2" t="n">
         <v>46044</v>
       </c>
       <c r="B71" t="n">
@@ -3254,7 +3268,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" s="2" t="n">
         <v>46045</v>
       </c>
       <c r="B72" t="n">
@@ -3268,7 +3282,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" s="2" t="n">
         <v>46048</v>
       </c>
       <c r="B73" t="n">
@@ -3282,7 +3296,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" s="2" t="n">
         <v>46049</v>
       </c>
       <c r="B74" t="n">
@@ -3296,7 +3310,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="B75" t="n">
@@ -3310,7 +3324,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" s="2" t="n">
         <v>46051</v>
       </c>
       <c r="B76" t="n">
@@ -3324,7 +3338,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" s="2" t="n">
         <v>46052</v>
       </c>
       <c r="B77" t="n">
@@ -3338,7 +3352,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" s="2" t="n">
         <v>46055</v>
       </c>
       <c r="B78" t="n">
@@ -3352,7 +3366,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" s="2" t="n">
         <v>46056</v>
       </c>
       <c r="B79" t="n">
@@ -3366,7 +3380,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" s="2" t="n">
         <v>46057</v>
       </c>
       <c r="B80" t="n">
@@ -3380,7 +3394,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" s="2" t="n">
         <v>46058</v>
       </c>
       <c r="B81" t="n">
@@ -3394,7 +3408,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" s="2" t="n">
         <v>46059</v>
       </c>
       <c r="B82" t="n">
@@ -3408,7 +3422,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" s="2" t="n">
         <v>46062</v>
       </c>
       <c r="B83" t="n">
@@ -3422,7 +3436,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="B84" t="n">
@@ -3436,7 +3450,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" s="2" t="n">
         <v>46064</v>
       </c>
       <c r="B85" t="n">
@@ -3450,7 +3464,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" s="2" t="n">
         <v>46065</v>
       </c>
       <c r="B86" t="n">
@@ -3464,7 +3478,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="B87" t="n">
@@ -3478,7 +3492,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" s="2" t="n">
         <v>46070</v>
       </c>
       <c r="B88" t="n">
@@ -3492,7 +3506,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" s="2" t="n">
         <v>46071</v>
       </c>
       <c r="B89" t="n">
@@ -3506,7 +3520,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" s="2" t="n">
         <v>46072</v>
       </c>
       <c r="B90" t="n">
@@ -3520,7 +3534,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" s="2" t="n">
         <v>46073</v>
       </c>
       <c r="B91" t="n">
@@ -3534,7 +3548,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" s="2" t="n">
         <v>46076</v>
       </c>
       <c r="B92" t="n">
@@ -3548,7 +3562,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" s="2" t="n">
         <v>46077</v>
       </c>
       <c r="B93" t="n">
@@ -3562,7 +3576,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" s="2" t="n">
         <v>46078</v>
       </c>
       <c r="B94" t="n">
@@ -3576,7 +3590,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" s="2" t="n">
         <v>46079</v>
       </c>
       <c r="B95" t="n">
@@ -3590,7 +3604,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="B96" t="n">
@@ -3604,7 +3618,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" s="2" t="n">
         <v>46083</v>
       </c>
       <c r="B97" t="n">
@@ -3618,7 +3632,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" s="2" t="n">
         <v>46084</v>
       </c>
       <c r="B98" t="n">
@@ -3632,7 +3646,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" s="2" t="n">
         <v>46085</v>
       </c>
       <c r="B99" t="n">
@@ -3646,7 +3660,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" s="2" t="n">
         <v>46086</v>
       </c>
       <c r="B100" t="n">
@@ -3660,7 +3674,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" s="2" t="n">
         <v>46087</v>
       </c>
       <c r="B101" t="n">
@@ -3674,7 +3688,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" s="2" t="n">
         <v>46090</v>
       </c>
       <c r="B102" t="n">
@@ -3688,7 +3702,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
+      <c r="A103" s="2" t="n">
         <v>46091</v>
       </c>
       <c r="B103" t="n">
@@ -3702,7 +3716,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
+      <c r="A104" s="2" t="n">
         <v>46092</v>
       </c>
       <c r="B104" t="n">
@@ -3716,7 +3730,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
+      <c r="A105" s="2" t="n">
         <v>46093</v>
       </c>
       <c r="B105" t="n">
@@ -3730,7 +3744,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
+      <c r="A106" s="2" t="n">
         <v>46094</v>
       </c>
       <c r="B106" t="n">
@@ -3744,7 +3758,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
+      <c r="A107" s="2" t="n">
         <v>46097</v>
       </c>
       <c r="B107" t="n">
@@ -3758,7 +3772,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
+      <c r="A108" s="2" t="n">
         <v>46098</v>
       </c>
       <c r="B108" t="n">
@@ -3772,7 +3786,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
+      <c r="A109" s="2" t="n">
         <v>46099</v>
       </c>
       <c r="B109" t="n">
@@ -3786,7 +3800,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="A110" s="2" t="n">
         <v>46100</v>
       </c>
       <c r="B110" t="n">
@@ -3800,7 +3814,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
+      <c r="A111" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="B111" t="n">
@@ -3814,7 +3828,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
+      <c r="A112" s="2" t="n">
         <v>46104</v>
       </c>
       <c r="B112" t="n">
@@ -3828,7 +3842,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
+      <c r="A113" s="2" t="n">
         <v>46105</v>
       </c>
       <c r="B113" t="n">
@@ -3842,7 +3856,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
+      <c r="A114" s="2" t="n">
         <v>46106</v>
       </c>
       <c r="B114" t="n">
@@ -3856,7 +3870,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
+      <c r="A115" s="2" t="n">
         <v>46107</v>
       </c>
       <c r="B115" t="n">
@@ -3870,7 +3884,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
+      <c r="A116" s="2" t="n">
         <v>46108</v>
       </c>
       <c r="B116" t="n">
@@ -3884,7 +3898,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
+      <c r="A117" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="B117" t="n">
@@ -3898,7 +3912,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
+      <c r="A118" s="2" t="n">
         <v>46112</v>
       </c>
       <c r="B118" t="n">
@@ -3912,7 +3926,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="n">
+      <c r="A119" s="2" t="n">
         <v>46113</v>
       </c>
       <c r="B119" t="n">
@@ -3926,7 +3940,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
+      <c r="A120" s="2" t="n">
         <v>46114</v>
       </c>
       <c r="B120" t="n">
@@ -3940,7 +3954,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="n">
+      <c r="A121" s="2" t="n">
         <v>46115</v>
       </c>
       <c r="B121" t="n">
@@ -3954,7 +3968,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="n">
+      <c r="A122" s="2" t="n">
         <v>46118</v>
       </c>
       <c r="B122" t="n">
@@ -3968,7 +3982,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="n">
+      <c r="A123" s="2" t="n">
         <v>46119</v>
       </c>
       <c r="B123" t="n">
@@ -3982,7 +3996,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="n">
+      <c r="A124" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="B124" t="n">
@@ -3996,7 +4010,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="n">
+      <c r="A125" s="2" t="n">
         <v>46121</v>
       </c>
       <c r="B125" t="n">
@@ -4010,7 +4024,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="n">
+      <c r="A126" s="2" t="n">
         <v>46122</v>
       </c>
       <c r="B126" t="n">
@@ -4024,7 +4038,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="n">
+      <c r="A127" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="B127" t="n">
@@ -4038,7 +4052,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="n">
+      <c r="A128" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="B128" t="n">
@@ -4052,7 +4066,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="n">
+      <c r="A129" s="2" t="n">
         <v>46127</v>
       </c>
       <c r="B129" t="n">
@@ -4066,7 +4080,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="n">
+      <c r="A130" s="2" t="n">
         <v>46128</v>
       </c>
       <c r="B130" t="n">
@@ -4080,7 +4094,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="n">
+      <c r="A131" s="2" t="n">
         <v>46129</v>
       </c>
       <c r="B131" t="n">
@@ -4094,7 +4108,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="n">
+      <c r="A132" s="2" t="n">
         <v>46132</v>
       </c>
       <c r="B132" t="n">
@@ -4108,7 +4122,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="n">
+      <c r="A133" s="2" t="n">
         <v>46133</v>
       </c>
       <c r="B133" t="n">
@@ -4122,7 +4136,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="n">
+      <c r="A134" s="2" t="n">
         <v>46134</v>
       </c>
       <c r="B134" t="n">
@@ -4136,7 +4150,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="n">
+      <c r="A135" s="2" t="n">
         <v>46135</v>
       </c>
       <c r="B135" t="n">
@@ -4150,7 +4164,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="n">
+      <c r="A136" s="2" t="n">
         <v>46136</v>
       </c>
       <c r="B136" t="n">
@@ -4164,7 +4178,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="n">
+      <c r="A137" s="2" t="n">
         <v>46139</v>
       </c>
       <c r="B137" t="n">
@@ -4178,7 +4192,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="1" t="n">
+      <c r="A138" s="2" t="n">
         <v>46140</v>
       </c>
       <c r="B138" t="n">
@@ -4192,7 +4206,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="1" t="n">
+      <c r="A139" s="2" t="n">
         <v>46141</v>
       </c>
       <c r="B139" t="n">
@@ -4206,7 +4220,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="1" t="n">
+      <c r="A140" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="B140" t="n">
@@ -4220,7 +4234,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="1" t="n">
+      <c r="A141" s="2" t="n">
         <v>46143</v>
       </c>
       <c r="B141" t="n">
@@ -4234,7 +4248,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="1" t="n">
+      <c r="A142" s="2" t="n">
         <v>46146</v>
       </c>
       <c r="B142" t="n">
@@ -4248,7 +4262,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="1" t="n">
+      <c r="A143" s="2" t="n">
         <v>46147</v>
       </c>
       <c r="B143" t="n">
@@ -4262,7 +4276,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="1" t="n">
+      <c r="A144" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="B144" t="n">
@@ -4276,7 +4290,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="1" t="n">
+      <c r="A145" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="B145" t="n">
@@ -4290,7 +4304,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="1" t="n">
+      <c r="A146" s="2" t="n">
         <v>46150</v>
       </c>
       <c r="B146" t="n">
@@ -4304,7 +4318,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="1" t="n">
+      <c r="A147" s="2" t="n">
         <v>46153</v>
       </c>
       <c r="B147" t="n">
@@ -4318,7 +4332,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="1" t="n">
+      <c r="A148" s="2" t="n">
         <v>46154</v>
       </c>
       <c r="B148" t="n">
@@ -4332,7 +4346,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="1" t="n">
+      <c r="A149" s="2" t="n">
         <v>46155</v>
       </c>
       <c r="B149" t="n">
@@ -4346,7 +4360,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="1" t="n">
+      <c r="A150" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="B150" t="n">
@@ -4360,7 +4374,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="1" t="n">
+      <c r="A151" s="2" t="n">
         <v>46157</v>
       </c>
       <c r="B151" t="n">
@@ -4374,7 +4388,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="1" t="n">
+      <c r="A152" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="B152" t="n">
@@ -4388,7 +4402,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="1" t="n">
+      <c r="A153" s="2" t="n">
         <v>46161</v>
       </c>
       <c r="B153" t="n">
@@ -4402,7 +4416,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="1" t="n">
+      <c r="A154" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="B154" t="n">
@@ -4416,7 +4430,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="1" t="n">
+      <c r="A155" s="2" t="n">
         <v>46163</v>
       </c>
       <c r="B155" t="n">
@@ -4430,7 +4444,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="1" t="n">
+      <c r="A156" s="2" t="n">
         <v>46164</v>
       </c>
       <c r="B156" t="n">
@@ -4444,7 +4458,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="1" t="n">
+      <c r="A157" s="2" t="n">
         <v>46168</v>
       </c>
       <c r="B157" t="n">
@@ -4458,7 +4472,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="1" t="n">
+      <c r="A158" s="2" t="n">
         <v>46169</v>
       </c>
       <c r="B158" t="n">
@@ -4472,7 +4486,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="1" t="n">
+      <c r="A159" s="2" t="n">
         <v>46170</v>
       </c>
       <c r="B159" t="n">
@@ -4486,7 +4500,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="1" t="n">
+      <c r="A160" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="B160" t="n">
@@ -4500,7 +4514,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="1" t="n">
+      <c r="A161" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="B161" t="n">
@@ -4514,7 +4528,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="1" t="n">
+      <c r="A162" s="2" t="n">
         <v>46175</v>
       </c>
       <c r="B162" t="n">
@@ -4528,7 +4542,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="1" t="n">
+      <c r="A163" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="B163" t="n">
@@ -4542,7 +4556,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="1" t="n">
+      <c r="A164" s="2" t="n">
         <v>46177</v>
       </c>
       <c r="B164" t="n">
@@ -4556,7 +4570,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="1" t="n">
+      <c r="A165" s="2" t="n">
         <v>46178</v>
       </c>
       <c r="B165" t="n">
@@ -4570,7 +4584,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="1" t="n">
+      <c r="A166" s="2" t="n">
         <v>46181</v>
       </c>
       <c r="B166" t="n">
@@ -4584,7 +4598,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="1" t="n">
+      <c r="A167" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="B167" t="n">
@@ -4598,7 +4612,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="1" t="n">
+      <c r="A168" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="B168" t="n">
@@ -4612,7 +4626,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="1" t="n">
+      <c r="A169" s="2" t="n">
         <v>46184</v>
       </c>
       <c r="B169" t="n">
@@ -4626,7 +4640,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="1" t="n">
+      <c r="A170" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="B170" t="n">
@@ -4640,7 +4654,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="1" t="n">
+      <c r="A171" s="2" t="n">
         <v>46188</v>
       </c>
       <c r="B171" t="n">
@@ -4654,7 +4668,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="1" t="n">
+      <c r="A172" s="2" t="n">
         <v>46189</v>
       </c>
       <c r="B172" t="n">
@@ -4668,7 +4682,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="1" t="n">
+      <c r="A173" s="2" t="n">
         <v>46190</v>
       </c>
       <c r="B173" t="n">
@@ -4682,7 +4696,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="1" t="n">
+      <c r="A174" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="B174" t="n">
@@ -4696,7 +4710,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="1" t="n">
+      <c r="A175" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="B175" t="n">
@@ -4710,7 +4724,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="1" t="n">
+      <c r="A176" s="2" t="n">
         <v>46196</v>
       </c>
       <c r="B176" t="n">
@@ -4724,7 +4738,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="1" t="n">
+      <c r="A177" s="2" t="n">
         <v>46197</v>
       </c>
       <c r="B177" t="n">
@@ -4738,7 +4752,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="1" t="n">
+      <c r="A178" s="2" t="n">
         <v>46198</v>
       </c>
       <c r="B178" t="n">
@@ -4752,7 +4766,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="1" t="n">
+      <c r="A179" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="B179" t="n">
@@ -4766,7 +4780,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="1" t="n">
+      <c r="A180" s="2" t="n">
         <v>46202</v>
       </c>
       <c r="B180" t="n">
@@ -4780,7 +4794,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="1" t="n">
+      <c r="A181" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="B181" t="n">
@@ -4794,7 +4808,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="1" t="n">
+      <c r="A182" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="B182" t="n">
@@ -4808,7 +4822,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="1" t="n">
+      <c r="A183" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="B183" t="n">
@@ -4822,7 +4836,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="1" t="n">
+      <c r="A184" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="B184" t="n">
@@ -4836,7 +4850,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="1" t="n">
+      <c r="A185" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="B185" t="n">
@@ -4850,7 +4864,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="1" t="n">
+      <c r="A186" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="B186" t="n">
@@ -4864,7 +4878,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="1" t="n">
+      <c r="A187" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="B187" t="n">
@@ -4878,7 +4892,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="1" t="n">
+      <c r="A188" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="B188" t="n">
@@ -4892,7 +4906,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="1" t="n">
+      <c r="A189" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="B189" t="n">
@@ -4906,7 +4920,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="1" t="n">
+      <c r="A190" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="B190" t="n">
@@ -4920,7 +4934,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="1" t="n">
+      <c r="A191" s="2" t="n">
         <v>46218</v>
       </c>
       <c r="B191" t="n">
@@ -4934,7 +4948,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="1" t="n">
+      <c r="A192" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="B192" t="n">
@@ -4948,7 +4962,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="1" t="n">
+      <c r="A193" s="2" t="n">
         <v>46220</v>
       </c>
       <c r="B193" t="n">
@@ -4962,7 +4976,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="1" t="n">
+      <c r="A194" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="B194" t="n">
@@ -4976,7 +4990,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="1" t="n">
+      <c r="A195" s="2" t="n">
         <v>46224</v>
       </c>
       <c r="B195" t="n">
@@ -4990,7 +5004,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="1" t="n">
+      <c r="A196" s="2" t="n">
         <v>46225</v>
       </c>
       <c r="B196" t="n">
@@ -5004,7 +5018,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="1" t="n">
+      <c r="A197" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="B197" t="n">
@@ -5018,7 +5032,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="1" t="n">
+      <c r="A198" s="2" t="n">
         <v>46227</v>
       </c>
       <c r="B198" t="n">
@@ -5032,7 +5046,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="1" t="n">
+      <c r="A199" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="B199" t="n">
@@ -5046,7 +5060,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="1" t="n">
+      <c r="A200" s="2" t="n">
         <v>46231</v>
       </c>
       <c r="B200" t="n">
@@ -5060,7 +5074,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="1" t="n">
+      <c r="A201" s="2" t="n">
         <v>46232</v>
       </c>
       <c r="B201" t="n">
@@ -5074,7 +5088,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="1" t="n">
+      <c r="A202" s="2" t="n">
         <v>46233</v>
       </c>
       <c r="B202" t="n">
@@ -5088,7 +5102,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="1" t="n">
+      <c r="A203" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B203" t="n">
@@ -5102,7 +5116,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="1" t="n">
+      <c r="A204" s="2" t="n">
         <v>46237</v>
       </c>
       <c r="B204" t="n">
@@ -5116,7 +5130,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="1" t="n">
+      <c r="A205" s="2" t="n">
         <v>46238</v>
       </c>
       <c r="B205" t="n">
@@ -5130,7 +5144,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="1" t="n">
+      <c r="A206" s="2" t="n">
         <v>46239</v>
       </c>
       <c r="B206" t="n">
@@ -5144,7 +5158,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="1" t="n">
+      <c r="A207" s="2" t="n">
         <v>46240</v>
       </c>
       <c r="B207" t="n">
@@ -5158,7 +5172,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="1" t="n">
+      <c r="A208" s="2" t="n">
         <v>46241</v>
       </c>
       <c r="B208" t="n">
@@ -5172,7 +5186,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="1" t="n">
+      <c r="A209" s="2" t="n">
         <v>46244</v>
       </c>
       <c r="B209" t="n">
@@ -5186,7 +5200,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="1" t="n">
+      <c r="A210" s="2" t="n">
         <v>46245</v>
       </c>
       <c r="B210" t="n">
@@ -5200,7 +5214,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="1" t="n">
+      <c r="A211" s="2" t="n">
         <v>46246</v>
       </c>
       <c r="B211" t="n">
@@ -5214,7 +5228,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="1" t="n">
+      <c r="A212" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="B212" t="n">
@@ -5228,7 +5242,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="1" t="n">
+      <c r="A213" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="B213" t="n">
@@ -5242,7 +5256,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="1" t="n">
+      <c r="A214" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="B214" t="n">
@@ -5256,7 +5270,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="1" t="n">
+      <c r="A215" s="2" t="n">
         <v>46252</v>
       </c>
       <c r="B215" t="n">
@@ -5270,7 +5284,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="1" t="n">
+      <c r="A216" s="2" t="n">
         <v>46253</v>
       </c>
       <c r="B216" t="n">
@@ -5284,7 +5298,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="1" t="n">
+      <c r="A217" s="2" t="n">
         <v>46254</v>
       </c>
       <c r="B217" t="n">
@@ -5298,7 +5312,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="1" t="n">
+      <c r="A218" s="2" t="n">
         <v>46255</v>
       </c>
       <c r="B218" t="n">
@@ -5312,7 +5326,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="1" t="n">
+      <c r="A219" s="2" t="n">
         <v>46258</v>
       </c>
       <c r="B219" t="n">
@@ -5326,7 +5340,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="1" t="n">
+      <c r="A220" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="B220" t="n">
@@ -5340,7 +5354,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="1" t="n">
+      <c r="A221" s="2" t="n">
         <v>46260</v>
       </c>
       <c r="B221" t="n">
@@ -5354,7 +5368,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="1" t="n">
+      <c r="A222" s="2" t="n">
         <v>46261</v>
       </c>
       <c r="B222" t="n">
@@ -5368,7 +5382,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="1" t="n">
+      <c r="A223" s="2" t="n">
         <v>46262</v>
       </c>
       <c r="B223" t="n">
@@ -5382,7 +5396,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="1" t="n">
+      <c r="A224" s="2" t="n">
         <v>46265</v>
       </c>
       <c r="B224" t="n">
@@ -5396,7 +5410,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="1" t="n">
+      <c r="A225" s="2" t="n">
         <v>46266</v>
       </c>
       <c r="B225" t="n">
@@ -5410,7 +5424,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="1" t="n">
+      <c r="A226" s="2" t="n">
         <v>46267</v>
       </c>
       <c r="B226" t="n">
@@ -5424,7 +5438,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="1" t="n">
+      <c r="A227" s="2" t="n">
         <v>46268</v>
       </c>
       <c r="B227" t="n">
@@ -5438,7 +5452,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="1" t="n">
+      <c r="A228" s="2" t="n">
         <v>46269</v>
       </c>
       <c r="B228" t="n">
@@ -5452,7 +5466,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="1" t="n">
+      <c r="A229" s="2" t="n">
         <v>46273</v>
       </c>
       <c r="B229" t="n">
@@ -5466,7 +5480,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="1" t="n">
+      <c r="A230" s="2" t="n">
         <v>46274</v>
       </c>
       <c r="B230" t="n">
@@ -5480,7 +5494,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="1" t="n">
+      <c r="A231" s="2" t="n">
         <v>46275</v>
       </c>
       <c r="B231" t="n">
@@ -5494,7 +5508,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="1" t="n">
+      <c r="A232" s="2" t="n">
         <v>46276</v>
       </c>
       <c r="B232" t="n">
@@ -5508,7 +5522,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="1" t="n">
+      <c r="A233" s="2" t="n">
         <v>46279</v>
       </c>
       <c r="B233" t="n">
@@ -5522,7 +5536,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="1" t="n">
+      <c r="A234" s="2" t="n">
         <v>46280</v>
       </c>
       <c r="B234" t="n">
@@ -5536,7 +5550,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="1" t="n">
+      <c r="A235" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="B235" t="n">
@@ -5550,7 +5564,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="1" t="n">
+      <c r="A236" s="2" t="n">
         <v>46282</v>
       </c>
       <c r="B236" t="n">
@@ -5564,7 +5578,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="1" t="n">
+      <c r="A237" s="2" t="n">
         <v>46283</v>
       </c>
       <c r="B237" t="n">
@@ -5578,7 +5592,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="1" t="n">
+      <c r="A238" s="2" t="n">
         <v>46286</v>
       </c>
       <c r="B238" t="n">
@@ -5592,7 +5606,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="1" t="n">
+      <c r="A239" s="2" t="n">
         <v>46287</v>
       </c>
       <c r="B239" t="n">
@@ -5606,7 +5620,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="1" t="n">
+      <c r="A240" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="B240" t="n">
@@ -5620,7 +5634,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="1" t="n">
+      <c r="A241" s="2" t="n">
         <v>46289</v>
       </c>
       <c r="B241" t="n">
@@ -5634,7 +5648,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="1" t="n">
+      <c r="A242" s="2" t="n">
         <v>46290</v>
       </c>
       <c r="B242" t="n">
@@ -5648,7 +5662,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="1" t="n">
+      <c r="A243" s="2" t="n">
         <v>46293</v>
       </c>
       <c r="B243" t="n">
@@ -5662,7 +5676,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="1" t="n">
+      <c r="A244" s="2" t="n">
         <v>46294</v>
       </c>
       <c r="B244" t="n">
@@ -5676,7 +5690,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="1" t="n">
+      <c r="A245" s="2" t="n">
         <v>46295</v>
       </c>
       <c r="B245" t="n">
@@ -5690,7 +5704,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="1" t="n">
+      <c r="A246" s="2" t="n">
         <v>46296</v>
       </c>
       <c r="B246" t="n">
@@ -5704,7 +5718,7 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="1" t="n">
+      <c r="A247" s="2" t="n">
         <v>46297</v>
       </c>
       <c r="B247" t="n">
@@ -5718,7 +5732,7 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="1" t="n">
+      <c r="A248" s="2" t="n">
         <v>46300</v>
       </c>
       <c r="B248" t="n">
@@ -5732,7 +5746,7 @@
       </c>
     </row>
     <row r="249">
-      <c r="A249" s="1" t="n">
+      <c r="A249" s="2" t="n">
         <v>46301</v>
       </c>
       <c r="B249" t="n">
@@ -5746,7 +5760,7 @@
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="1" t="n">
+      <c r="A250" s="2" t="n">
         <v>46302</v>
       </c>
       <c r="B250" t="n">
@@ -5760,7 +5774,7 @@
       </c>
     </row>
     <row r="251">
-      <c r="A251" s="1" t="n">
+      <c r="A251" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B251" t="n">
@@ -5788,49 +5802,49 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>1y-3m</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>2y-1y</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>5y-2y</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>10y-5y</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>5y-1y</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>fly 2*1y-3m-2y</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>fly 2*2y-1y-5y</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>fly 2*5y-2y-10y</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>1y-3m</t>
         </is>
@@ -5861,7 +5875,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>2y-1y</t>
         </is>
@@ -5892,7 +5906,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>5y-2y</t>
         </is>
@@ -5923,7 +5937,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>10y-5y</t>
         </is>
@@ -5954,7 +5968,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>5y-1y</t>
         </is>
@@ -5985,7 +5999,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>fly 2*1y-3m-2y</t>
         </is>
@@ -6016,7 +6030,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>fly 2*2y-1y-5y</t>
         </is>
@@ -6047,7 +6061,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>fly 2*5y-2y-10y</t>
         </is>
@@ -6092,49 +6106,49 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>1y-3m</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>2y-1y</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>5y-2y</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>10y-5y</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>5y-1y</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>fly 2*1y-3m-2y</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>fly 2*2y-1y-5y</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>fly 2*5y-2y-10y</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>1y-3m</t>
         </is>
@@ -6165,7 +6179,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>2y-1y</t>
         </is>
@@ -6196,7 +6210,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>5y-2y</t>
         </is>
@@ -6227,7 +6241,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>10y-5y</t>
         </is>
@@ -6258,7 +6272,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>5y-1y</t>
         </is>
@@ -6289,7 +6303,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>fly 2*1y-3m-2y</t>
         </is>
@@ -6320,7 +6334,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>fly 2*2y-1y-5y</t>
         </is>
@@ -6351,7 +6365,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>fly 2*5y-2y-10y</t>
         </is>
@@ -6396,49 +6410,49 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>1y-3m</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>2y-1y</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>5y-2y</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>10y-5y</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>5y-1y</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>fly 2*1y-3m-2y</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>fly 2*2y-1y-5y</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>fly 2*5y-2y-10y</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>1y-3m</t>
         </is>
@@ -6469,7 +6483,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>2y-1y</t>
         </is>
@@ -6500,7 +6514,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>5y-2y</t>
         </is>
@@ -6531,7 +6545,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>10y-5y</t>
         </is>
@@ -6562,7 +6576,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>5y-1y</t>
         </is>
@@ -6593,7 +6607,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>fly 2*1y-3m-2y</t>
         </is>
@@ -6624,7 +6638,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>fly 2*2y-1y-5y</t>
         </is>
@@ -6655,7 +6669,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>fly 2*5y-2y-10y</t>
         </is>

</xml_diff>